<commit_message>
Add Max to the Name column in ridley.xlsx.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ridley.xlsx
+++ b/ridley.xlsx
@@ -413,13 +413,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
           <t>ridley</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Max</t>
         </is>
       </c>
     </row>

</xml_diff>